<commit_message>
Verison 2 antes de agregar comentarios
</commit_message>
<xml_diff>
--- a/reportes/reporte_admin.xlsx
+++ b/reportes/reporte_admin.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,6 +506,126 @@
       </c>
       <c r="J2" t="n">
         <v>416.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ryuk</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>08/03/2026 17:25</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pijamas</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>270000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>53865</v>
+      </c>
+      <c r="H3" t="n">
+        <v>337365</v>
+      </c>
+      <c r="I3" t="n">
+        <v>81000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>347.12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ryuk</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08/03/2026 17:37</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>9500</v>
+      </c>
+      <c r="H4" t="n">
+        <v>59500</v>
+      </c>
+      <c r="I4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J4" t="n">
+        <v>347.12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ryuk</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/03/2026 20:19</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>26</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Inteligente</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>260000</v>
+      </c>
+      <c r="G5" t="n">
+        <v>49400</v>
+      </c>
+      <c r="H5" t="n">
+        <v>309400</v>
+      </c>
+      <c r="I5" t="n">
+        <v>78000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>520.6799999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version terminada Faltan los archivos de reportes
</commit_message>
<xml_diff>
--- a/reportes/reporte_admin.xlsx
+++ b/reportes/reporte_admin.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,6 +628,206 @@
         <v>520.6799999999999</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pepe</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10/03/2026 22:20</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>interior</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Inteligente</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>39900</v>
+      </c>
+      <c r="H6" t="n">
+        <v>249900</v>
+      </c>
+      <c r="I6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>520.6799999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/03/2026 22:50</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Inteligente</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G7" t="n">
+        <v>38000</v>
+      </c>
+      <c r="H7" t="n">
+        <v>238000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>368.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/03/2026 22:53</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>pijamas</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Inteligente</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>19950</v>
+      </c>
+      <c r="H8" t="n">
+        <v>124950</v>
+      </c>
+      <c r="I8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>442.56</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Miska</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/03/2026 23:16</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Inteligente</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G9" t="n">
+        <v>38000</v>
+      </c>
+      <c r="H9" t="n">
+        <v>238000</v>
+      </c>
+      <c r="I9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J9" t="n">
+        <v>147.52</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Miska</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10/03/2026 23:18</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>40</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>vestidos</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Inteligente</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G10" t="n">
+        <v>79800</v>
+      </c>
+      <c r="H10" t="n">
+        <v>499800</v>
+      </c>
+      <c r="I10" t="n">
+        <v>120000</v>
+      </c>
+      <c r="J10" t="n">
+        <v>147.52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>